<commit_message>
nazia kamran kashif novels added
</commit_message>
<xml_diff>
--- a/add_new_novel.xlsx
+++ b/add_new_novel.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18350" windowHeight="5750"/>
+    <workbookView windowWidth="18350" windowHeight="6470"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
   <si>
     <t>Titles</t>
   </si>
@@ -35,16 +35,43 @@
     <t>Links</t>
   </si>
   <si>
-    <t>Mahe Darakhshan novel by fatima laghari</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/drive/folders/1MFnuGT1O3vVMlJRfQ9C4qz1vTvI-0oGY?fbclid=PAZXh0bgNhZW0CMTEAc3J0YwZhcHBfaWQMMjU2MjgxMDQwNTU4AAGn0rvmQ5QSqs2bHKjQQ66bSDRjHrS767nE0uA4dwSrT65Wl-T5w_btZ3lxw-M_aem_0jEW2Uznk2mzvZF8ROCFCQ</t>
-  </si>
-  <si>
-    <t>Mahe Darakhshan by fatima laghari</t>
-  </si>
-  <si>
-    <t>Mahe Darakhshan novel Folder</t>
+    <t>Makli by Nazia Kamran Kashif</t>
+  </si>
+  <si>
+    <t>https://www.urdunovelbanks.com/2026/01/makli-novel-by-nazia-kamran-kashif-read.html</t>
+  </si>
+  <si>
+    <t>Shaka by Nazia kamran Kashif</t>
+  </si>
+  <si>
+    <t>https://www.urdunovelbanks.com/2026/01/shaka-novel-by-nazia-kamran-kashif-read.html</t>
+  </si>
+  <si>
+    <t>Ishq Zaad by Nazia Kamran Kashif</t>
+  </si>
+  <si>
+    <t>https://www.urdunovelbanks.com/2026/01/ishq-zaad-novel-by-nazia-kamran-kashif.html</t>
+  </si>
+  <si>
+    <t>Bermuda Triangle By Nazia Kamran Kashif</t>
+  </si>
+  <si>
+    <t>https://www.urdunovelbanks.com/2026/01/bermuda-triangle-by-nazia-kamran-kashif.html</t>
+  </si>
+  <si>
+    <t>Bermuda Triangle complete novel</t>
+  </si>
+  <si>
+    <t>Barmuda Triangle novel</t>
+  </si>
+  <si>
+    <t>Barmuda Triangle PDF</t>
+  </si>
+  <si>
+    <t>Ishqzaad by Nazia Kamran Kashif</t>
+  </si>
+  <si>
+    <t>Ishqzaad novel  by Nazia Kamran Kashif</t>
   </si>
 </sst>
 </file>
@@ -57,7 +84,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -68,22 +95,30 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
       <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -553,140 +588,140 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
@@ -1007,8 +1042,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="1"/>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="50.0909090909091" style="1" customWidth="1"/>
     <col min="2" max="2" width="47.1818181818182" style="1" customWidth="1"/>
@@ -1016,42 +1051,96 @@
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:2">
+    <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:2">
+    <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>3</v>
+      <c r="B3" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" spans="1:2">
+    <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>3</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" s="2" customFormat="1" spans="1:2">
+      <c r="A10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="https://drive.google.com/drive/folders/1MFnuGT1O3vVMlJRfQ9C4qz1vTvI-0oGY?fbclid=PAZXh0bgNhZW0CMTEAc3J0YwZhcHBfaWQMMjU2MjgxMDQwNTU4AAGn0rvmQ5QSqs2bHKjQQ66bSDRjHrS767nE0uA4dwSrT65Wl-T5w_btZ3lxw-M_aem_0jEW2Uznk2mzvZF8ROCFCQ" tooltip="https://drive.google.com/drive/folders/1MFnuGT1O3vVMlJRfQ9C4qz1vTvI-0oGY?fbclid=PAZXh0bgNhZW0CMTEAc3J0YwZhcHBfaWQMMjU2MjgxMDQwNTU4AAGn0rvmQ5QSqs2bHKjQQ66bSDRjHrS767nE0uA4dwSrT65Wl-T5w_btZ3lxw-M_aem_0jEW2Uznk2mzvZF8ROCFCQ"/>
-    <hyperlink ref="B3" r:id="rId1" display="https://drive.google.com/drive/folders/1MFnuGT1O3vVMlJRfQ9C4qz1vTvI-0oGY?fbclid=PAZXh0bgNhZW0CMTEAc3J0YwZhcHBfaWQMMjU2MjgxMDQwNTU4AAGn0rvmQ5QSqs2bHKjQQ66bSDRjHrS767nE0uA4dwSrT65Wl-T5w_btZ3lxw-M_aem_0jEW2Uznk2mzvZF8ROCFCQ"/>
-    <hyperlink ref="B4" r:id="rId1" display="https://drive.google.com/drive/folders/1MFnuGT1O3vVMlJRfQ9C4qz1vTvI-0oGY?fbclid=PAZXh0bgNhZW0CMTEAc3J0YwZhcHBfaWQMMjU2MjgxMDQwNTU4AAGn0rvmQ5QSqs2bHKjQQ66bSDRjHrS767nE0uA4dwSrT65Wl-T5w_btZ3lxw-M_aem_0jEW2Uznk2mzvZF8ROCFCQ"/>
+    <hyperlink ref="B2" r:id="rId1" display="https://www.urdunovelbanks.com/2026/01/makli-novel-by-nazia-kamran-kashif-read.html"/>
+    <hyperlink ref="B3" r:id="rId2" display="https://www.urdunovelbanks.com/2026/01/shaka-novel-by-nazia-kamran-kashif-read.html"/>
+    <hyperlink ref="B4" r:id="rId3" display="https://www.urdunovelbanks.com/2026/01/ishq-zaad-novel-by-nazia-kamran-kashif.html"/>
+    <hyperlink ref="B5" r:id="rId4" display="https://www.urdunovelbanks.com/2026/01/bermuda-triangle-by-nazia-kamran-kashif.html"/>
+    <hyperlink ref="B6" r:id="rId4" display="https://www.urdunovelbanks.com/2026/01/bermuda-triangle-by-nazia-kamran-kashif.html"/>
+    <hyperlink ref="B7" r:id="rId4" display="https://www.urdunovelbanks.com/2026/01/bermuda-triangle-by-nazia-kamran-kashif.html"/>
+    <hyperlink ref="B8" r:id="rId4" display="https://www.urdunovelbanks.com/2026/01/bermuda-triangle-by-nazia-kamran-kashif.html"/>
+    <hyperlink ref="B9" r:id="rId3" display="https://www.urdunovelbanks.com/2026/01/ishq-zaad-novel-by-nazia-kamran-kashif.html"/>
+    <hyperlink ref="B10" r:id="rId3" display="https://www.urdunovelbanks.com/2026/01/ishq-zaad-novel-by-nazia-kamran-kashif.html"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>